<commit_message>
Excel sheet updates for BMX
</commit_message>
<xml_diff>
--- a/data/source_files/1. BA - IE3 - AC.xlsx
+++ b/data/source_files/1. BA - IE3 - AC.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1168" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1169" uniqueCount="202">
   <si>
     <t>Motor Type</t>
   </si>
@@ -155,10 +155,10 @@
     <t>(Amps)</t>
   </si>
   <si>
+    <t>Italy</t>
+  </si>
+  <si>
     <t>1.8 / 1.1</t>
-  </si>
-  <si>
-    <t>Italy</t>
   </si>
   <si>
     <t>3.5 / 2.0</t>
@@ -2684,14 +2684,14 @@
       <c r="C9" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="D9" s="15">
-        <v>90.1</v>
+      <c r="D9" s="15" t="s">
+        <v>42</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G9" s="14" t="s">
         <v>44</v>
@@ -2762,13 +2762,13 @@
         <v>64</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E10" s="16">
         <v>1415</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G10" s="14">
         <v>1415</v>
@@ -2839,13 +2839,13 @@
         <v>66</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E11" s="16">
         <v>2.6</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G11" s="14">
         <v>5.06</v>
@@ -3291,13 +3291,13 @@
         <v>78</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E17" s="21">
         <v>4.5</v>
       </c>
       <c r="F17" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G17" s="14">
         <v>5.6</v>
@@ -3368,13 +3368,13 @@
         <v>80</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E18" s="21">
         <v>3.5</v>
       </c>
       <c r="F18" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G18" s="14">
         <v>3.1</v>
@@ -3445,13 +3445,13 @@
         <v>82</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E19" s="22">
         <v>3.6</v>
       </c>
       <c r="F19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G19" s="22">
         <v>3.2</v>
@@ -3460,55 +3460,55 @@
         <v>3.9</v>
       </c>
       <c r="I19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K19" s="22">
         <v>4.5</v>
       </c>
       <c r="L19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="T19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="V19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Y19" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" customHeight="1" spans="1:25">
@@ -3522,13 +3522,13 @@
         <v>1</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E20" s="25">
         <v>77.8</v>
       </c>
       <c r="F20" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G20" s="14">
         <v>82.5</v>
@@ -3597,13 +3597,13 @@
         <v>0.75</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E21" s="28">
         <v>77.2</v>
       </c>
       <c r="F21" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G21" s="14">
         <v>82.8</v>
@@ -3672,13 +3672,13 @@
         <v>0.5</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E22" s="31">
         <v>73.8</v>
       </c>
       <c r="F22" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G22" s="14">
         <v>81.2</v>
@@ -3749,13 +3749,13 @@
         <v>1</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E23" s="32">
         <v>0.63</v>
       </c>
       <c r="F23" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G23" s="33">
         <v>0.67</v>
@@ -3824,13 +3824,13 @@
         <v>0.75</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E24" s="34">
         <v>0.53</v>
       </c>
       <c r="F24" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G24" s="33">
         <v>0.6</v>
@@ -3899,13 +3899,13 @@
         <v>0.5</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E25" s="35">
         <v>0.41</v>
       </c>
       <c r="F25" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G25" s="33">
         <v>0.47</v>
@@ -4051,70 +4051,70 @@
         <v>88</v>
       </c>
       <c r="D27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="T27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="V27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Y27" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28" customHeight="1" spans="1:25">
@@ -4126,70 +4126,70 @@
         <v>89</v>
       </c>
       <c r="D28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="T28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="V28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Y28" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29" customHeight="1" spans="1:25">
@@ -4203,70 +4203,70 @@
         <v>91</v>
       </c>
       <c r="D29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="T29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="V29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Y29" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="30" customHeight="1" spans="1:25">
@@ -4736,70 +4736,70 @@
         <v>119</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="T36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="V36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Y36" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37" customHeight="1" spans="1:25">
@@ -4853,28 +4853,28 @@
         <v>123</v>
       </c>
       <c r="R37" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S37" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="T37" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U37" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="V37" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W37" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X37" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Y37" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="38" customHeight="1" spans="1:25">
@@ -5374,34 +5374,34 @@
         <v>140</v>
       </c>
       <c r="P44" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q44" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R44" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S44" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="T44" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U44" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="V44" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W44" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X44" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Y44" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="45" customHeight="1" spans="1:25">
@@ -5542,13 +5542,13 @@
         <v>147</v>
       </c>
       <c r="V46" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W46" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X46" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Y46" s="20" t="s">
         <v>148</v>
@@ -5696,13 +5696,13 @@
         <v>157</v>
       </c>
       <c r="V48" s="45" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W48" s="45" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X48" s="45" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Y48" s="45" t="s">
         <v>148</v>
@@ -6954,70 +6954,70 @@
       </c>
       <c r="C65" s="10"/>
       <c r="D65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="T65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="V65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Y65" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="66" customHeight="1" spans="1:25">
@@ -7029,70 +7029,70 @@
       </c>
       <c r="C66" s="10"/>
       <c r="D66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="T66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="V66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Y66" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="67" customHeight="1" spans="1:25">
@@ -7104,70 +7104,70 @@
       </c>
       <c r="C67" s="10"/>
       <c r="D67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="T67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="V67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Y67" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="68" customHeight="1" spans="1:25">
@@ -7179,70 +7179,70 @@
       </c>
       <c r="C68" s="10"/>
       <c r="D68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="T68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="V68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Y68" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="69" customHeight="1" spans="1:25">
@@ -7254,70 +7254,70 @@
       </c>
       <c r="C69" s="10"/>
       <c r="D69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="T69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="V69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Y69" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="70" customHeight="1" spans="1:25">
@@ -7329,70 +7329,70 @@
       </c>
       <c r="C70" s="10"/>
       <c r="D70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="T70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="V70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Y70" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="71" customHeight="1" spans="1:25">
@@ -7404,70 +7404,70 @@
       </c>
       <c r="C71" s="10"/>
       <c r="D71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="T71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="V71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Y71" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Motor overall over just slight modifications only to be altered
</commit_message>
<xml_diff>
--- a/data/source_files/1. BA - IE3 - AC.xlsx
+++ b/data/source_files/1. BA - IE3 - AC.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1169" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1128" uniqueCount="200">
   <si>
     <t>Motor Type</t>
   </si>
@@ -161,6 +161,9 @@
     <t>1.8 / 1.1</t>
   </si>
   <si>
+    <t>2.43 / 1.41</t>
+  </si>
+  <si>
     <t>3.5 / 2.0</t>
   </si>
   <si>
@@ -173,16 +176,16 @@
     <t>8.3 / 4.8</t>
   </si>
   <si>
-    <t>13.3 / 7.7</t>
-  </si>
-  <si>
-    <t>19.1 / 11.0</t>
-  </si>
-  <si>
-    <t>25.8 / 14.9</t>
-  </si>
-  <si>
-    <t>38.6 / 22.3</t>
+    <t>14 / 8.4</t>
+  </si>
+  <si>
+    <t>19.1 / 11.1</t>
+  </si>
+  <si>
+    <t>26.0 / 15.0</t>
+  </si>
+  <si>
+    <t>37.7 / 21.8</t>
   </si>
   <si>
     <t>52.3 / 30.2</t>
@@ -191,7 +194,7 @@
     <t>64.2 / 37.1</t>
   </si>
   <si>
-    <t>72.1 / 41.7</t>
+    <t>72.5 / 41.7</t>
   </si>
   <si>
     <t>92.0 / 53.2</t>
@@ -200,7 +203,7 @@
     <t>114.5 / 66.2</t>
   </si>
   <si>
-    <t>137.2 / 79.3</t>
+    <t>137.9 / 79.3</t>
   </si>
   <si>
     <t>167.1 / 96.6</t>
@@ -495,9 +498,6 @@
     <t>NDE</t>
   </si>
   <si>
-    <t>9309Z</t>
-  </si>
-  <si>
     <t>6314Z</t>
   </si>
   <si>
@@ -589,9 +589,6 @@
   </si>
   <si>
     <t>M4</t>
-  </si>
-  <si>
-    <t>M6</t>
   </si>
   <si>
     <t>M8</t>
@@ -711,9 +708,6 @@
     <t>IS : 12615 / IEC 60034-1</t>
   </si>
   <si>
-    <t>IS : 12615 / IEC 60034-0</t>
-  </si>
-  <si>
     <t>Vibration severity grade</t>
   </si>
   <si>
@@ -820,14 +814,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="180" formatCode="0.0"/>
+    <numFmt numFmtId="181" formatCode="0.0_ "/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -866,6 +861,13 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1028,7 +1030,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1212,6 +1214,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1425,152 +1433,152 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="179" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1635,7 +1643,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="181" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2691,64 +2708,64 @@
         <v>43</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="K9" s="14" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="N9" s="14" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="O9" s="14" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="P9" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="Q9" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="R9" s="14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="S9" s="14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="T9" s="14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="U9" s="14" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="V9" s="14" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="W9" s="14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="X9" s="14" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Y9" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" customHeight="1" spans="1:25">
@@ -2756,10 +2773,10 @@
         <v>10</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D10" s="15" t="s">
         <v>42</v>
@@ -2767,8 +2784,8 @@
       <c r="E10" s="16">
         <v>1415</v>
       </c>
-      <c r="F10" s="15" t="s">
-        <v>42</v>
+      <c r="F10" s="15">
+        <v>1408</v>
       </c>
       <c r="G10" s="14">
         <v>1415</v>
@@ -2783,7 +2800,7 @@
         <v>1440</v>
       </c>
       <c r="K10" s="14">
-        <v>1450</v>
+        <v>1445</v>
       </c>
       <c r="L10" s="14">
         <v>1457</v>
@@ -2833,10 +2850,10 @@
         <v>11</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D11" s="15" t="s">
         <v>42</v>
@@ -2844,14 +2861,14 @@
       <c r="E11" s="16">
         <v>2.6</v>
       </c>
-      <c r="F11" s="15" t="s">
-        <v>42</v>
+      <c r="F11" s="15">
+        <v>3.7</v>
       </c>
       <c r="G11" s="14">
-        <v>5.06</v>
+        <v>5.1</v>
       </c>
       <c r="H11" s="14">
-        <v>7.37</v>
+        <v>7.4</v>
       </c>
       <c r="I11" s="14">
         <v>10</v>
@@ -2860,16 +2877,16 @@
         <v>14.5</v>
       </c>
       <c r="K11" s="14">
-        <v>24.2</v>
+        <v>26.4</v>
       </c>
       <c r="L11" s="17">
-        <v>36</v>
+        <v>36.1</v>
       </c>
       <c r="M11" s="14">
-        <v>49.2</v>
+        <v>49.3</v>
       </c>
       <c r="N11" s="14">
-        <v>71.5</v>
+        <v>71.9</v>
       </c>
       <c r="O11" s="14">
         <v>97.4</v>
@@ -2890,7 +2907,7 @@
         <v>290.4</v>
       </c>
       <c r="U11" s="14">
-        <v>354.9</v>
+        <v>354.88</v>
       </c>
       <c r="V11" s="14">
         <v>481.3</v>
@@ -2910,74 +2927,74 @@
         <v>12</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C12" s="10"/>
       <c r="D12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="L12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="M12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="N12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="O12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="P12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="R12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="S12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="T12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="U12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="V12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="W12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="X12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Y12" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" customHeight="1" spans="1:25">
@@ -2985,74 +3002,74 @@
         <v>13</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="L13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="M13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="P13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="R13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="S13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="T13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="U13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="V13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="W13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="X13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Y13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" customHeight="1" spans="1:25">
@@ -3060,74 +3077,74 @@
         <v>14</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C14" s="10"/>
       <c r="D14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="L14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="P14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="R14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="S14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="T14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="U14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="V14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="W14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="X14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Y14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" customHeight="1" spans="1:25">
@@ -3135,74 +3152,74 @@
         <v>15</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="L15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="M15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="N15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="P15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="Q15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="R15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="S15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="T15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="U15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="V15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="W15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="X15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="Y15" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" customHeight="1" spans="1:25">
@@ -3210,74 +3227,74 @@
         <v>16</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="M16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="N16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="P16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Q16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="R16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="S16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="T16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="U16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="V16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="W16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="X16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Y16" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" customHeight="1" spans="1:25">
@@ -3285,64 +3302,64 @@
         <v>17</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D17" s="20" t="s">
         <v>42</v>
       </c>
       <c r="E17" s="21">
-        <v>4.5</v>
-      </c>
-      <c r="F17" s="20" t="s">
-        <v>42</v>
+        <v>4.9</v>
+      </c>
+      <c r="F17" s="20">
+        <v>6.1</v>
       </c>
       <c r="G17" s="14">
-        <v>5.6</v>
+        <v>11.2</v>
       </c>
       <c r="H17" s="14">
-        <v>5.7</v>
-      </c>
-      <c r="I17" s="14">
-        <v>6.2</v>
+        <v>14.8</v>
+      </c>
+      <c r="I17" s="22">
+        <v>21</v>
       </c>
       <c r="J17" s="17">
-        <v>7</v>
+        <v>33.6</v>
       </c>
       <c r="K17" s="14">
-        <v>7.1</v>
+        <v>66.4</v>
       </c>
       <c r="L17" s="14">
-        <v>7.6</v>
+        <v>86.6</v>
       </c>
       <c r="M17" s="14">
-        <v>7.9</v>
+        <v>109.5</v>
       </c>
       <c r="N17" s="14">
-        <v>9.1</v>
+        <v>128.6</v>
       </c>
       <c r="O17" s="14">
-        <v>9.1</v>
+        <v>274.8</v>
       </c>
       <c r="P17" s="14">
-        <v>9.1</v>
-      </c>
-      <c r="Q17" s="14">
-        <v>8.6</v>
+        <v>337.6</v>
+      </c>
+      <c r="Q17" s="22">
+        <v>358</v>
       </c>
       <c r="R17" s="14">
-        <v>8.4</v>
+        <v>447</v>
       </c>
       <c r="S17" s="14">
-        <v>8.5</v>
-      </c>
-      <c r="T17" s="14">
-        <v>8.8</v>
+        <v>563</v>
+      </c>
+      <c r="T17" s="22">
+        <v>377</v>
       </c>
       <c r="U17" s="14">
-        <v>9.8</v>
+        <v>946.7</v>
       </c>
       <c r="V17" s="14">
         <v>7.6</v>
@@ -3362,64 +3379,64 @@
         <v>18</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D18" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="E18" s="21">
-        <v>3.5</v>
-      </c>
-      <c r="F18" s="20" t="s">
-        <v>42</v>
+      <c r="E18" s="23">
+        <v>9</v>
+      </c>
+      <c r="F18" s="20">
+        <v>8.5</v>
       </c>
       <c r="G18" s="14">
-        <v>3.1</v>
+        <v>15.8</v>
       </c>
       <c r="H18" s="14">
-        <v>3.4</v>
-      </c>
-      <c r="I18" s="14">
-        <v>3.5</v>
+        <v>25.2</v>
+      </c>
+      <c r="I18" s="22">
+        <v>35</v>
       </c>
       <c r="J18" s="14">
-        <v>2.9</v>
-      </c>
-      <c r="K18" s="14">
-        <v>3.7</v>
+        <v>42.1</v>
+      </c>
+      <c r="K18" s="22">
+        <v>122</v>
       </c>
       <c r="L18" s="14">
-        <v>3.5</v>
+        <v>122.7</v>
       </c>
       <c r="M18" s="14">
-        <v>3.3</v>
+        <v>172.6</v>
       </c>
       <c r="N18" s="14">
-        <v>3.8</v>
-      </c>
-      <c r="O18" s="14">
-        <v>3.5</v>
+        <v>172.6</v>
+      </c>
+      <c r="O18" s="22">
+        <v>340</v>
       </c>
       <c r="P18" s="14">
-        <v>3.5</v>
-      </c>
-      <c r="Q18" s="14">
-        <v>4.3</v>
+        <v>299.5</v>
+      </c>
+      <c r="Q18" s="22">
+        <v>404</v>
       </c>
       <c r="R18" s="14">
-        <v>2.9</v>
+        <v>563</v>
       </c>
       <c r="S18" s="14">
-        <v>2.7</v>
-      </c>
-      <c r="T18" s="14">
-        <v>2.8</v>
-      </c>
-      <c r="U18" s="14">
-        <v>3.2</v>
+        <v>644</v>
+      </c>
+      <c r="T18" s="22">
+        <v>800</v>
+      </c>
+      <c r="U18" s="22">
+        <v>1135</v>
       </c>
       <c r="V18" s="14">
         <v>2.2</v>
@@ -3439,64 +3456,64 @@
         <v>19</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D19" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="E19" s="22">
-        <v>3.6</v>
-      </c>
-      <c r="F19" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="G19" s="22">
-        <v>3.2</v>
-      </c>
-      <c r="H19" s="22">
-        <v>3.9</v>
-      </c>
-      <c r="I19" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="J19" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="K19" s="22">
-        <v>4.5</v>
-      </c>
-      <c r="L19" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="M19" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="N19" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="O19" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="P19" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q19" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="R19" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="S19" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="T19" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="U19" s="20" t="s">
-        <v>42</v>
+      <c r="E19" s="24">
+        <v>10.1</v>
+      </c>
+      <c r="F19" s="20">
+        <v>1.7</v>
+      </c>
+      <c r="G19" s="24">
+        <v>16.2</v>
+      </c>
+      <c r="H19" s="24">
+        <v>28.9</v>
+      </c>
+      <c r="I19" s="25">
+        <v>38</v>
+      </c>
+      <c r="J19" s="25">
+        <v>45</v>
+      </c>
+      <c r="K19" s="24">
+        <v>132.5</v>
+      </c>
+      <c r="L19" s="25">
+        <v>130</v>
+      </c>
+      <c r="M19" s="20">
+        <v>167.6</v>
+      </c>
+      <c r="N19" s="20">
+        <v>186.9</v>
+      </c>
+      <c r="O19" s="25">
+        <v>379</v>
+      </c>
+      <c r="P19" s="20">
+        <v>311.4</v>
+      </c>
+      <c r="Q19" s="25">
+        <v>413</v>
+      </c>
+      <c r="R19" s="20">
+        <v>640</v>
+      </c>
+      <c r="S19" s="20">
+        <v>664</v>
+      </c>
+      <c r="T19" s="25">
+        <v>820</v>
+      </c>
+      <c r="U19" s="25">
+        <v>1242</v>
       </c>
       <c r="V19" s="20" t="s">
         <v>42</v>
@@ -3515,20 +3532,20 @@
       <c r="A20" s="8">
         <v>20</v>
       </c>
-      <c r="B20" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="C20" s="24">
+      <c r="B20" s="26" t="s">
+        <v>84</v>
+      </c>
+      <c r="C20" s="27">
         <v>1</v>
       </c>
       <c r="D20" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="E20" s="25">
+      <c r="E20" s="28">
         <v>77.8</v>
       </c>
-      <c r="F20" s="20" t="s">
-        <v>42</v>
+      <c r="F20" s="20">
+        <v>77.1</v>
       </c>
       <c r="G20" s="14">
         <v>82.5</v>
@@ -3543,7 +3560,7 @@
         <v>86.7</v>
       </c>
       <c r="K20" s="14">
-        <v>88.8</v>
+        <v>88.6</v>
       </c>
       <c r="L20" s="14">
         <v>89.6</v>
@@ -3570,7 +3587,7 @@
         <v>93.9</v>
       </c>
       <c r="T20" s="14">
-        <v>94.2</v>
+        <v>93.1</v>
       </c>
       <c r="U20" s="14">
         <v>94.6</v>
@@ -3592,18 +3609,18 @@
       <c r="A21" s="8">
         <v>21</v>
       </c>
-      <c r="B21" s="26"/>
-      <c r="C21" s="27">
+      <c r="B21" s="29"/>
+      <c r="C21" s="30">
         <v>0.75</v>
       </c>
       <c r="D21" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="E21" s="28">
+      <c r="E21" s="31">
         <v>77.2</v>
       </c>
-      <c r="F21" s="20" t="s">
-        <v>42</v>
+      <c r="F21" s="20">
+        <v>76.4</v>
       </c>
       <c r="G21" s="14">
         <v>82.8</v>
@@ -3618,7 +3635,7 @@
         <v>87</v>
       </c>
       <c r="K21" s="14">
-        <v>88.9</v>
+        <v>88.8</v>
       </c>
       <c r="L21" s="14">
         <v>91.1</v>
@@ -3645,7 +3662,7 @@
         <v>94.4</v>
       </c>
       <c r="T21" s="14">
-        <v>94.7</v>
+        <v>93.6</v>
       </c>
       <c r="U21" s="14">
         <v>95.1</v>
@@ -3667,18 +3684,18 @@
       <c r="A22" s="8">
         <v>22</v>
       </c>
-      <c r="B22" s="29"/>
-      <c r="C22" s="30">
+      <c r="B22" s="32"/>
+      <c r="C22" s="33">
         <v>0.5</v>
       </c>
       <c r="D22" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="E22" s="31">
+      <c r="E22" s="34">
         <v>73.8</v>
       </c>
-      <c r="F22" s="20" t="s">
-        <v>42</v>
+      <c r="F22" s="20">
+        <v>73.5</v>
       </c>
       <c r="G22" s="14">
         <v>81.2</v>
@@ -3720,7 +3737,7 @@
         <v>91.9</v>
       </c>
       <c r="T22" s="14">
-        <v>92.2</v>
+        <v>92.8</v>
       </c>
       <c r="U22" s="14">
         <v>92.6</v>
@@ -3742,76 +3759,76 @@
       <c r="A23" s="8">
         <v>23</v>
       </c>
-      <c r="B23" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="C23" s="24">
+      <c r="B23" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" s="27">
         <v>1</v>
       </c>
       <c r="D23" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="E23" s="32">
+      <c r="E23" s="35">
         <v>0.63</v>
       </c>
-      <c r="F23" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="G23" s="33">
+      <c r="F23" s="20">
+        <v>0.72</v>
+      </c>
+      <c r="G23" s="36">
         <v>0.67</v>
       </c>
-      <c r="H23" s="33">
+      <c r="H23" s="36">
         <v>0.73</v>
       </c>
-      <c r="I23" s="33">
+      <c r="I23" s="36">
         <v>0.74</v>
       </c>
-      <c r="J23" s="33">
+      <c r="J23" s="36">
         <v>0.76</v>
       </c>
-      <c r="K23" s="33">
-        <v>0.76</v>
-      </c>
-      <c r="L23" s="33">
-        <v>0.8</v>
-      </c>
-      <c r="M23" s="33">
+      <c r="K23" s="36">
+        <v>0.77</v>
+      </c>
+      <c r="L23" s="36">
         <v>0.82</v>
       </c>
-      <c r="N23" s="33">
+      <c r="M23" s="36">
+        <v>0.82</v>
+      </c>
+      <c r="N23" s="36">
         <v>0.78</v>
       </c>
-      <c r="O23" s="33">
+      <c r="O23" s="36">
         <v>0.78</v>
       </c>
-      <c r="P23" s="33">
+      <c r="P23" s="36">
         <v>0.78</v>
       </c>
-      <c r="Q23" s="33">
+      <c r="Q23" s="36">
         <v>0.82</v>
       </c>
-      <c r="R23" s="33">
+      <c r="R23" s="36">
         <v>0.87</v>
       </c>
-      <c r="S23" s="33">
+      <c r="S23" s="36">
         <v>0.86</v>
       </c>
-      <c r="T23" s="33">
+      <c r="T23" s="36">
         <v>0.87</v>
       </c>
-      <c r="U23" s="33">
+      <c r="U23" s="36">
         <v>0.87</v>
       </c>
-      <c r="V23" s="33">
+      <c r="V23" s="36">
         <v>0.83</v>
       </c>
-      <c r="W23" s="33">
+      <c r="W23" s="36">
         <v>0.84</v>
       </c>
-      <c r="X23" s="33">
+      <c r="X23" s="36">
         <v>0.86</v>
       </c>
-      <c r="Y23" s="33">
+      <c r="Y23" s="36">
         <v>0.86</v>
       </c>
     </row>
@@ -3819,74 +3836,74 @@
       <c r="A24" s="8">
         <v>24</v>
       </c>
-      <c r="B24" s="26"/>
-      <c r="C24" s="27">
+      <c r="B24" s="29"/>
+      <c r="C24" s="30">
         <v>0.75</v>
       </c>
       <c r="D24" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="E24" s="34">
+      <c r="E24" s="37">
         <v>0.53</v>
       </c>
-      <c r="F24" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="G24" s="33">
+      <c r="F24" s="20">
+        <v>0.61</v>
+      </c>
+      <c r="G24" s="36">
         <v>0.6</v>
       </c>
-      <c r="H24" s="33">
+      <c r="H24" s="36">
         <v>0.64</v>
       </c>
-      <c r="I24" s="33">
+      <c r="I24" s="36">
         <v>0.64</v>
       </c>
-      <c r="J24" s="33">
+      <c r="J24" s="36">
         <v>0.67</v>
       </c>
-      <c r="K24" s="33">
-        <v>0.68</v>
-      </c>
-      <c r="L24" s="33">
+      <c r="K24" s="36">
+        <v>0.67</v>
+      </c>
+      <c r="L24" s="36">
+        <v>0.77</v>
+      </c>
+      <c r="M24" s="36">
+        <v>0.72</v>
+      </c>
+      <c r="N24" s="36">
         <v>0.74</v>
       </c>
-      <c r="M24" s="33">
+      <c r="O24" s="36">
+        <v>0.71</v>
+      </c>
+      <c r="P24" s="36">
+        <v>0.72</v>
+      </c>
+      <c r="Q24" s="36">
         <v>0.75</v>
       </c>
-      <c r="N24" s="33">
-        <v>0.71</v>
-      </c>
-      <c r="O24" s="33">
-        <v>0.71</v>
-      </c>
-      <c r="P24" s="33">
-        <v>0.72</v>
-      </c>
-      <c r="Q24" s="33">
-        <v>0.73</v>
-      </c>
-      <c r="R24" s="33">
+      <c r="R24" s="36">
         <v>0.84</v>
       </c>
-      <c r="S24" s="33">
+      <c r="S24" s="36">
         <v>0.77</v>
       </c>
-      <c r="T24" s="33">
+      <c r="T24" s="36">
+        <v>0.84</v>
+      </c>
+      <c r="U24" s="36">
         <v>0.78</v>
       </c>
-      <c r="U24" s="33">
-        <v>0.78</v>
-      </c>
-      <c r="V24" s="33">
+      <c r="V24" s="36">
         <v>0.79</v>
       </c>
-      <c r="W24" s="33">
+      <c r="W24" s="36">
         <v>0.75</v>
       </c>
-      <c r="X24" s="33">
+      <c r="X24" s="36">
         <v>0.77</v>
       </c>
-      <c r="Y24" s="33">
+      <c r="Y24" s="36">
         <v>0.77</v>
       </c>
     </row>
@@ -3894,74 +3911,74 @@
       <c r="A25" s="8">
         <v>25</v>
       </c>
-      <c r="B25" s="29"/>
-      <c r="C25" s="30">
+      <c r="B25" s="32"/>
+      <c r="C25" s="33">
         <v>0.5</v>
       </c>
       <c r="D25" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="E25" s="35">
+      <c r="E25" s="38">
         <v>0.41</v>
       </c>
-      <c r="F25" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="G25" s="33">
+      <c r="F25" s="20">
+        <v>0.48</v>
+      </c>
+      <c r="G25" s="36">
         <v>0.47</v>
       </c>
-      <c r="H25" s="33">
+      <c r="H25" s="36">
         <v>0.5</v>
       </c>
-      <c r="I25" s="33">
+      <c r="I25" s="36">
         <v>0.5</v>
       </c>
-      <c r="J25" s="33">
+      <c r="J25" s="36">
         <v>0.54</v>
       </c>
-      <c r="K25" s="33">
-        <v>0.54</v>
-      </c>
-      <c r="L25" s="33">
+      <c r="K25" s="36">
+        <v>0.52</v>
+      </c>
+      <c r="L25" s="36">
+        <v>0.65</v>
+      </c>
+      <c r="M25" s="36">
+        <v>0.61</v>
+      </c>
+      <c r="N25" s="36">
         <v>0.62</v>
       </c>
-      <c r="M25" s="33">
+      <c r="O25" s="36">
+        <v>0.59</v>
+      </c>
+      <c r="P25" s="36">
+        <v>0.59</v>
+      </c>
+      <c r="Q25" s="36">
         <v>0.63</v>
       </c>
-      <c r="N25" s="33">
-        <v>0.59</v>
-      </c>
-      <c r="O25" s="33">
-        <v>0.59</v>
-      </c>
-      <c r="P25" s="33">
-        <v>0.59</v>
-      </c>
-      <c r="Q25" s="33">
-        <v>0.68</v>
-      </c>
-      <c r="R25" s="33">
+      <c r="R25" s="36">
         <v>0.75</v>
       </c>
-      <c r="S25" s="33">
+      <c r="S25" s="36">
         <v>0.72</v>
       </c>
-      <c r="T25" s="33">
+      <c r="T25" s="36">
+        <v>0.76</v>
+      </c>
+      <c r="U25" s="36">
         <v>0.73</v>
       </c>
-      <c r="U25" s="33">
-        <v>0.73</v>
-      </c>
-      <c r="V25" s="33">
+      <c r="V25" s="36">
         <v>0.69</v>
       </c>
-      <c r="W25" s="33">
+      <c r="W25" s="36">
         <v>0.7</v>
       </c>
-      <c r="X25" s="33">
+      <c r="X25" s="36">
         <v>0.72</v>
       </c>
-      <c r="Y25" s="33">
+      <c r="Y25" s="36">
         <v>0.72</v>
       </c>
     </row>
@@ -3970,85 +3987,85 @@
         <v>26</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C26" s="10"/>
       <c r="D26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="L26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="M26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="N26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="P26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="R26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="S26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="T26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="U26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="V26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="W26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="X26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Y26" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="27" customHeight="1" spans="1:25">
       <c r="A27" s="8">
         <v>27</v>
       </c>
-      <c r="B27" s="23" t="s">
-        <v>87</v>
+      <c r="B27" s="26" t="s">
+        <v>88</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D27" s="20" t="s">
         <v>42</v>
@@ -4121,9 +4138,9 @@
       <c r="A28" s="8">
         <v>28</v>
       </c>
-      <c r="B28" s="29"/>
-      <c r="C28" s="36" t="s">
-        <v>89</v>
+      <c r="B28" s="32"/>
+      <c r="C28" s="39" t="s">
+        <v>90</v>
       </c>
       <c r="D28" s="20" t="s">
         <v>42</v>
@@ -4197,10 +4214,10 @@
         <v>29</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D29" s="20" t="s">
         <v>42</v>
@@ -4273,137 +4290,137 @@
       <c r="A30" s="8">
         <v>30</v>
       </c>
-      <c r="B30" s="23" t="s">
-        <v>92</v>
-      </c>
-      <c r="C30" s="37" t="s">
+      <c r="B30" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="D30" s="38" t="s">
+      <c r="C30" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="E30" s="38" t="s">
-        <v>94</v>
+      <c r="D30" s="41" t="s">
+        <v>95</v>
+      </c>
+      <c r="E30" s="41" t="s">
+        <v>95</v>
       </c>
       <c r="F30" s="14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G30" s="14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H30" s="14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I30" s="14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J30" s="14" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K30" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L30" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="M30" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="N30" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="O30" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="P30" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q30" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="R30" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="S30" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="T30" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="U30" s="14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="V30" s="14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="W30" s="14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="X30" s="14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Y30" s="14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="31" customHeight="1" spans="1:25">
       <c r="A31" s="8">
         <v>31</v>
       </c>
-      <c r="B31" s="29"/>
+      <c r="B31" s="32"/>
       <c r="C31" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E31" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G31" s="14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H31" s="14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I31" s="14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J31" s="14" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K31" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L31" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="M31" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="N31" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="O31" s="14" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="P31" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q31" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="R31" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="S31" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T31" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="U31" s="14" t="s">
         <v>108</v>
@@ -4415,10 +4432,10 @@
         <v>108</v>
       </c>
       <c r="X31" s="14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Y31" s="14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="32" customHeight="1" spans="1:25">
@@ -4577,7 +4594,7 @@
       <c r="A34" s="8">
         <v>34</v>
       </c>
-      <c r="B34" s="23" t="s">
+      <c r="B34" s="26" t="s">
         <v>113</v>
       </c>
       <c r="C34" s="10" t="s">
@@ -4654,8 +4671,8 @@
       <c r="A35" s="8">
         <v>35</v>
       </c>
-      <c r="B35" s="29"/>
-      <c r="C35" s="36" t="s">
+      <c r="B35" s="32"/>
+      <c r="C35" s="39" t="s">
         <v>117</v>
       </c>
       <c r="D35" s="14" t="s">
@@ -4738,56 +4755,56 @@
       <c r="D36" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="E36" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="F36" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="G36" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="H36" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="I36" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="J36" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K36" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="L36" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="M36" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="N36" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="O36" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="P36" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q36" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="R36" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="S36" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="T36" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="U36" s="15" t="s">
-        <v>42</v>
+      <c r="E36" s="15">
+        <v>10.5</v>
+      </c>
+      <c r="F36" s="15">
+        <v>15</v>
+      </c>
+      <c r="G36" s="15">
+        <v>17</v>
+      </c>
+      <c r="H36" s="15">
+        <v>21</v>
+      </c>
+      <c r="I36" s="15">
+        <v>24</v>
+      </c>
+      <c r="J36" s="15">
+        <v>36</v>
+      </c>
+      <c r="K36" s="15">
+        <v>50</v>
+      </c>
+      <c r="L36" s="15">
+        <v>86</v>
+      </c>
+      <c r="M36" s="15">
+        <v>95</v>
+      </c>
+      <c r="N36" s="15">
+        <v>160</v>
+      </c>
+      <c r="O36" s="15">
+        <v>175</v>
+      </c>
+      <c r="P36" s="15">
+        <v>250</v>
+      </c>
+      <c r="Q36" s="15">
+        <v>250</v>
+      </c>
+      <c r="R36" s="15">
+        <v>300</v>
+      </c>
+      <c r="S36" s="15">
+        <v>450</v>
+      </c>
+      <c r="T36" s="15">
+        <v>465</v>
+      </c>
+      <c r="U36" s="15">
+        <v>665</v>
       </c>
       <c r="V36" s="15" t="s">
         <v>42</v>
@@ -4853,16 +4870,16 @@
         <v>123</v>
       </c>
       <c r="R37" s="20" t="s">
-        <v>42</v>
+        <v>123</v>
       </c>
       <c r="S37" s="20" t="s">
-        <v>42</v>
+        <v>123</v>
       </c>
       <c r="T37" s="20" t="s">
-        <v>42</v>
+        <v>123</v>
       </c>
       <c r="U37" s="20" t="s">
-        <v>42</v>
+        <v>123</v>
       </c>
       <c r="V37" s="20" t="s">
         <v>42</v>
@@ -4885,70 +4902,70 @@
         <v>124</v>
       </c>
       <c r="C38" s="10"/>
-      <c r="D38" s="39" t="s">
+      <c r="D38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="E38" s="39" t="s">
+      <c r="E38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="F38" s="39" t="s">
+      <c r="F38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="G38" s="39" t="s">
+      <c r="G38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="H38" s="39" t="s">
+      <c r="H38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="I38" s="39" t="s">
+      <c r="I38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="J38" s="39" t="s">
+      <c r="J38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="K38" s="39" t="s">
+      <c r="K38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="L38" s="39" t="s">
+      <c r="L38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="M38" s="39" t="s">
+      <c r="M38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="N38" s="39" t="s">
+      <c r="N38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="O38" s="39" t="s">
+      <c r="O38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="P38" s="39" t="s">
+      <c r="P38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="Q38" s="39" t="s">
+      <c r="Q38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="R38" s="39" t="s">
+      <c r="R38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="S38" s="39" t="s">
+      <c r="S38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="T38" s="39" t="s">
+      <c r="T38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="U38" s="39" t="s">
+      <c r="U38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="V38" s="39" t="s">
+      <c r="V38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="W38" s="39" t="s">
+      <c r="W38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="X38" s="39" t="s">
+      <c r="X38" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="Y38" s="39" t="s">
+      <c r="Y38" s="42" t="s">
         <v>125</v>
       </c>
     </row>
@@ -4960,70 +4977,70 @@
         <v>126</v>
       </c>
       <c r="C39" s="10"/>
-      <c r="D39" s="39" t="s">
+      <c r="D39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="E39" s="39" t="s">
+      <c r="E39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="F39" s="39" t="s">
+      <c r="F39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="G39" s="39" t="s">
+      <c r="G39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="H39" s="39" t="s">
+      <c r="H39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="I39" s="39" t="s">
+      <c r="I39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="J39" s="39" t="s">
+      <c r="J39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="K39" s="39" t="s">
+      <c r="K39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="L39" s="39" t="s">
+      <c r="L39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="M39" s="39" t="s">
+      <c r="M39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="N39" s="39" t="s">
+      <c r="N39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="O39" s="39" t="s">
+      <c r="O39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="P39" s="39" t="s">
+      <c r="P39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="Q39" s="39" t="s">
+      <c r="Q39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="R39" s="39" t="s">
+      <c r="R39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="S39" s="39" t="s">
+      <c r="S39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="T39" s="39" t="s">
+      <c r="T39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="U39" s="39" t="s">
+      <c r="U39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="V39" s="39" t="s">
+      <c r="V39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="W39" s="39" t="s">
+      <c r="W39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="X39" s="39" t="s">
+      <c r="X39" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="Y39" s="39" t="s">
+      <c r="Y39" s="42" t="s">
         <v>127</v>
       </c>
     </row>
@@ -5035,70 +5052,70 @@
         <v>128</v>
       </c>
       <c r="C40" s="10"/>
-      <c r="D40" s="39" t="s">
+      <c r="D40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="E40" s="39" t="s">
+      <c r="E40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="F40" s="39" t="s">
+      <c r="F40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="G40" s="39" t="s">
+      <c r="G40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="H40" s="39" t="s">
+      <c r="H40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="I40" s="39" t="s">
+      <c r="I40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="J40" s="39" t="s">
+      <c r="J40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="K40" s="39" t="s">
+      <c r="K40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="L40" s="39" t="s">
+      <c r="L40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="M40" s="39" t="s">
+      <c r="M40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="N40" s="39" t="s">
+      <c r="N40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="O40" s="39" t="s">
+      <c r="O40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="P40" s="39" t="s">
+      <c r="P40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="Q40" s="39" t="s">
+      <c r="Q40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="R40" s="39" t="s">
+      <c r="R40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="S40" s="39" t="s">
+      <c r="S40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="T40" s="39" t="s">
+      <c r="T40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="U40" s="39" t="s">
+      <c r="U40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="V40" s="39" t="s">
+      <c r="V40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="W40" s="39" t="s">
+      <c r="W40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="X40" s="39" t="s">
+      <c r="X40" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="Y40" s="39" t="s">
+      <c r="Y40" s="42" t="s">
         <v>125</v>
       </c>
     </row>
@@ -5109,7 +5126,7 @@
       <c r="B41" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="C41" s="40" t="s">
+      <c r="C41" s="43" t="s">
         <v>130</v>
       </c>
       <c r="D41" s="14" t="s">
@@ -5293,28 +5310,28 @@
         <v>135</v>
       </c>
       <c r="N43" s="14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="O43" s="14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P43" s="14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="Q43" s="14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="R43" s="14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="S43" s="14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="T43" s="14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="U43" s="14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="V43" s="14" t="s">
         <v>136</v>
@@ -5362,16 +5379,16 @@
         <v>138</v>
       </c>
       <c r="L44" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="M44" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="N44" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="O44" s="14" t="s">
         <v>139</v>
-      </c>
-      <c r="M44" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="N44" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="O44" s="14" t="s">
-        <v>140</v>
       </c>
       <c r="P44" s="20" t="s">
         <v>42</v>
@@ -5409,7 +5426,7 @@
         <v>45</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C45" s="10"/>
       <c r="D45" s="16">
@@ -5483,12 +5500,12 @@
       <c r="A46" s="8">
         <v>46</v>
       </c>
-      <c r="B46" s="41" t="s">
-        <v>142</v>
+      <c r="B46" s="44" t="s">
+        <v>141</v>
       </c>
       <c r="C46" s="19"/>
       <c r="D46" s="14" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E46" s="14" t="s">
         <v>143</v>
@@ -5500,69 +5517,69 @@
         <v>143</v>
       </c>
       <c r="H46" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="I46" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="J46" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="K46" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="L46" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="I46" s="14" t="s">
+      <c r="M46" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="J46" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="K46" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="L46" s="14" t="s">
+      <c r="N46" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="M46" s="14" t="s">
+      <c r="O46" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="N46" s="14" t="s">
+      <c r="P46" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q46" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="R46" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="S46" s="14" t="s">
         <v>146</v>
       </c>
-      <c r="O46" s="14" t="s">
+      <c r="T46" s="14" t="s">
         <v>146</v>
       </c>
-      <c r="P46" s="14" t="s">
+      <c r="U46" s="14" t="s">
         <v>146</v>
       </c>
-      <c r="Q46" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="R46" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="S46" s="14" t="s">
+      <c r="V46" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="W46" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="X46" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y46" s="20" t="s">
         <v>147</v>
-      </c>
-      <c r="T46" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="U46" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="V46" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="W46" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="X46" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y46" s="20" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="47" customHeight="1" spans="1:25">
       <c r="A47" s="8">
         <v>47</v>
       </c>
-      <c r="B47" s="41" t="s">
+      <c r="B47" s="44" t="s">
+        <v>148</v>
+      </c>
+      <c r="C47" s="19" t="s">
         <v>149</v>
-      </c>
-      <c r="C47" s="19" t="s">
-        <v>150</v>
       </c>
       <c r="D47" s="21">
         <v>1</v>
@@ -5635,465 +5652,465 @@
       <c r="A48" s="8">
         <v>48</v>
       </c>
-      <c r="B48" s="42" t="s">
+      <c r="B48" s="45" t="s">
+        <v>150</v>
+      </c>
+      <c r="C48" s="46" t="s">
         <v>151</v>
       </c>
-      <c r="C48" s="43" t="s">
+      <c r="D48" s="47" t="s">
         <v>152</v>
       </c>
-      <c r="D48" s="44" t="s">
+      <c r="E48" s="47" t="s">
+        <v>152</v>
+      </c>
+      <c r="F48" s="47" t="s">
+        <v>152</v>
+      </c>
+      <c r="G48" s="47" t="s">
+        <v>152</v>
+      </c>
+      <c r="H48" s="47" t="s">
         <v>153</v>
       </c>
-      <c r="E48" s="44" t="s">
+      <c r="I48" s="47" t="s">
         <v>153</v>
       </c>
-      <c r="F48" s="44" t="s">
+      <c r="J48" s="47" t="s">
         <v>153</v>
       </c>
-      <c r="G48" s="44" t="s">
+      <c r="K48" s="47" t="s">
         <v>153</v>
       </c>
-      <c r="H48" s="44" t="s">
+      <c r="L48" s="47" t="s">
         <v>154</v>
       </c>
-      <c r="I48" s="44" t="s">
+      <c r="M48" s="47" t="s">
         <v>154</v>
       </c>
-      <c r="J48" s="44" t="s">
-        <v>154</v>
-      </c>
-      <c r="K48" s="44" t="s">
-        <v>154</v>
-      </c>
-      <c r="L48" s="44" t="s">
+      <c r="N48" s="47" t="s">
         <v>155</v>
       </c>
-      <c r="M48" s="44" t="s">
+      <c r="O48" s="47" t="s">
         <v>155</v>
       </c>
-      <c r="N48" s="44" t="s">
+      <c r="P48" s="47" t="s">
+        <v>155</v>
+      </c>
+      <c r="Q48" s="47" t="s">
+        <v>155</v>
+      </c>
+      <c r="R48" s="47" t="s">
+        <v>155</v>
+      </c>
+      <c r="S48" s="47" t="s">
         <v>156</v>
       </c>
-      <c r="O48" s="44" t="s">
+      <c r="T48" s="47" t="s">
         <v>156</v>
       </c>
-      <c r="P48" s="44" t="s">
+      <c r="U48" s="47" t="s">
         <v>156</v>
       </c>
-      <c r="Q48" s="44" t="s">
-        <v>156</v>
-      </c>
-      <c r="R48" s="44" t="s">
-        <v>156</v>
-      </c>
-      <c r="S48" s="44" t="s">
-        <v>157</v>
-      </c>
-      <c r="T48" s="44" t="s">
-        <v>157</v>
-      </c>
-      <c r="U48" s="44" t="s">
-        <v>157</v>
-      </c>
-      <c r="V48" s="45" t="s">
-        <v>42</v>
-      </c>
-      <c r="W48" s="45" t="s">
-        <v>42</v>
-      </c>
-      <c r="X48" s="45" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y48" s="45" t="s">
-        <v>148</v>
+      <c r="V48" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="W48" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="X48" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y48" s="48" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="49" customHeight="1" spans="1:26">
       <c r="A49" s="8">
         <v>49</v>
       </c>
-      <c r="B49" s="41" t="s">
+      <c r="B49" s="44" t="s">
+        <v>157</v>
+      </c>
+      <c r="C49" s="19" t="s">
         <v>158</v>
       </c>
-      <c r="C49" s="19" t="s">
+      <c r="D49" s="49" t="s">
         <v>159</v>
       </c>
-      <c r="D49" s="46" t="s">
+      <c r="E49" s="49" t="s">
+        <v>159</v>
+      </c>
+      <c r="F49" s="49" t="s">
+        <v>159</v>
+      </c>
+      <c r="G49" s="49" t="s">
+        <v>159</v>
+      </c>
+      <c r="H49" s="49" t="s">
         <v>160</v>
       </c>
-      <c r="E49" s="46" t="s">
+      <c r="I49" s="49" t="s">
         <v>160</v>
       </c>
-      <c r="F49" s="46" t="s">
+      <c r="J49" s="49" t="s">
         <v>160</v>
       </c>
-      <c r="G49" s="46" t="s">
+      <c r="K49" s="49" t="s">
         <v>160</v>
       </c>
-      <c r="H49" s="46" t="s">
+      <c r="L49" s="49" t="s">
         <v>161</v>
       </c>
-      <c r="I49" s="46" t="s">
+      <c r="M49" s="49" t="s">
         <v>161</v>
       </c>
-      <c r="J49" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="K49" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="L49" s="46" t="s">
+      <c r="N49" s="49" t="s">
         <v>162</v>
       </c>
-      <c r="M49" s="46" t="s">
+      <c r="O49" s="49" t="s">
         <v>162</v>
       </c>
-      <c r="N49" s="46" t="s">
+      <c r="P49" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q49" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="R49" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="S49" s="49" t="s">
         <v>163</v>
       </c>
-      <c r="O49" s="46" t="s">
+      <c r="T49" s="49" t="s">
         <v>163</v>
       </c>
-      <c r="P49" s="46" t="s">
+      <c r="U49" s="49" t="s">
         <v>163</v>
       </c>
-      <c r="Q49" s="46" t="s">
-        <v>163</v>
-      </c>
-      <c r="R49" s="46" t="s">
-        <v>163</v>
-      </c>
-      <c r="S49" s="46" t="s">
+      <c r="V49" s="20" t="s">
         <v>164</v>
       </c>
-      <c r="T49" s="46" t="s">
+      <c r="W49" s="20" t="s">
         <v>164</v>
       </c>
-      <c r="U49" s="46" t="s">
+      <c r="X49" s="20" t="s">
         <v>164</v>
       </c>
-      <c r="V49" s="20" t="s">
-        <v>165</v>
-      </c>
-      <c r="W49" s="20" t="s">
-        <v>165</v>
-      </c>
-      <c r="X49" s="20" t="s">
-        <v>165</v>
-      </c>
       <c r="Y49" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="50" customHeight="1" spans="1:26">
       <c r="A50" s="8">
         <v>50</v>
       </c>
-      <c r="B50" s="41" t="s">
-        <v>166</v>
+      <c r="B50" s="44" t="s">
+        <v>165</v>
       </c>
       <c r="C50" s="19"/>
       <c r="D50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="L50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="M50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="N50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="O50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="P50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="Q50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="S50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="V50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="W50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="X50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="Y50" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="51" customHeight="1" spans="1:26">
       <c r="A51" s="8">
         <v>51</v>
       </c>
-      <c r="B51" s="41" t="s">
-        <v>168</v>
+      <c r="B51" s="44" t="s">
+        <v>167</v>
       </c>
       <c r="C51" s="19"/>
       <c r="D51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="I51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="M51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="N51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="P51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="Q51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="T51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="U51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="V51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="W51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="X51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="Y51" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="52" s="4" customFormat="1" customHeight="1" spans="1:26">
       <c r="A52" s="8">
         <v>52</v>
       </c>
-      <c r="B52" s="47" t="s">
+      <c r="B52" s="50" t="s">
+        <v>169</v>
+      </c>
+      <c r="C52" s="51"/>
+      <c r="D52" s="52" t="s">
         <v>170</v>
       </c>
-      <c r="C52" s="48"/>
-      <c r="D52" s="49" t="s">
+      <c r="E52" s="52" t="s">
         <v>171</v>
       </c>
-      <c r="E52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="F52" s="49" t="s">
-        <v>173</v>
-      </c>
-      <c r="G52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="H52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="I52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="J52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="K52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="L52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="M52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="N52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="O52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="P52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="Q52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="R52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="S52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="T52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="U52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="V52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="W52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="X52" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="Y52" s="49" t="s">
-        <v>172</v>
+      <c r="F52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="G52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="H52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="I52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="J52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="K52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="L52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="M52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="N52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="O52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="P52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="Q52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="R52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="S52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="T52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="U52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="V52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="W52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="X52" s="52" t="s">
+        <v>171</v>
+      </c>
+      <c r="Y52" s="52" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="53" customHeight="1" spans="1:26">
       <c r="A53" s="8">
         <v>53</v>
       </c>
-      <c r="B53" s="41" t="s">
-        <v>174</v>
+      <c r="B53" s="44" t="s">
+        <v>172</v>
       </c>
       <c r="C53" s="19"/>
-      <c r="D53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="E53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="F53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="G53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="H53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="I53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="J53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="K53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="L53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="M53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="N53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="O53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="P53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="Q53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="R53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="S53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="T53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="U53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="V53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="W53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="X53" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="Y53" s="50" t="s">
-        <v>175</v>
+      <c r="D53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="E53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="F53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="G53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="H53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="I53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="J53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="K53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="L53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="M53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="N53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="O53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="P53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="Q53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="R53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="S53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="T53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="U53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="V53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="W53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="X53" s="53" t="s">
+        <v>173</v>
+      </c>
+      <c r="Y53" s="53" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="54" customHeight="1" spans="1:26">
       <c r="A54" s="8">
         <v>54</v>
       </c>
-      <c r="B54" s="41" t="s">
-        <v>176</v>
+      <c r="B54" s="44" t="s">
+        <v>174</v>
       </c>
       <c r="C54" s="19" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D54" s="21">
         <v>45</v>
@@ -6104,61 +6121,61 @@
       <c r="F54" s="21">
         <v>47</v>
       </c>
-      <c r="G54" s="50">
+      <c r="G54" s="53">
         <v>47</v>
       </c>
-      <c r="H54" s="50">
+      <c r="H54" s="53">
         <v>55</v>
       </c>
-      <c r="I54" s="50">
+      <c r="I54" s="53">
         <v>55</v>
       </c>
-      <c r="J54" s="50">
+      <c r="J54" s="53">
         <v>57</v>
       </c>
-      <c r="K54" s="50">
+      <c r="K54" s="53">
         <v>61</v>
       </c>
-      <c r="L54" s="50">
+      <c r="L54" s="53">
         <v>62</v>
       </c>
-      <c r="M54" s="50">
+      <c r="M54" s="53">
         <v>62</v>
       </c>
-      <c r="N54" s="50">
+      <c r="N54" s="53">
         <v>63</v>
       </c>
-      <c r="O54" s="50">
+      <c r="O54" s="53">
         <v>63</v>
       </c>
-      <c r="P54" s="50">
+      <c r="P54" s="53">
         <v>64</v>
       </c>
-      <c r="Q54" s="50">
+      <c r="Q54" s="53">
         <v>64</v>
       </c>
-      <c r="R54" s="50">
+      <c r="R54" s="53">
         <v>66</v>
       </c>
-      <c r="S54" s="50">
+      <c r="S54" s="53">
         <v>68</v>
       </c>
-      <c r="T54" s="50">
+      <c r="T54" s="53">
         <v>68</v>
       </c>
-      <c r="U54" s="50">
+      <c r="U54" s="53">
         <v>70</v>
       </c>
-      <c r="V54" s="50">
+      <c r="V54" s="53">
         <v>70</v>
       </c>
-      <c r="W54" s="50">
+      <c r="W54" s="53">
         <v>70</v>
       </c>
-      <c r="X54" s="50">
+      <c r="X54" s="53">
         <v>70</v>
       </c>
-      <c r="Y54" s="50">
+      <c r="Y54" s="53">
         <v>70</v>
       </c>
     </row>
@@ -6166,88 +6183,88 @@
       <c r="A55" s="8">
         <v>55</v>
       </c>
-      <c r="B55" s="41" t="s">
+      <c r="B55" s="44" t="s">
+        <v>176</v>
+      </c>
+      <c r="C55" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="D55" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="C55" s="19" t="s">
-        <v>179</v>
-      </c>
-      <c r="D55" s="14" t="s">
-        <v>180</v>
-      </c>
       <c r="E55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="I55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="J55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="K55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="L55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="M55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="N55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="O55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="P55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="Q55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="R55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="S55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="T55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="U55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="V55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="W55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="X55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="Y55" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="56" customHeight="1" spans="1:26">
       <c r="A56" s="8">
         <v>56</v>
       </c>
-      <c r="B56" s="41" t="s">
-        <v>181</v>
+      <c r="B56" s="44" t="s">
+        <v>179</v>
       </c>
       <c r="C56" s="19" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D56" s="14">
         <v>415</v>
@@ -6320,86 +6337,86 @@
       <c r="A57" s="8">
         <v>57</v>
       </c>
-      <c r="B57" s="41" t="s">
-        <v>183</v>
+      <c r="B57" s="44" t="s">
+        <v>181</v>
       </c>
       <c r="C57" s="19"/>
       <c r="D57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="F57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="I57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="J57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="K57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="L57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="M57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="N57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="O57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="P57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="Q57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="R57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="S57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="T57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="U57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="V57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="W57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="X57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="Y57" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="58" customHeight="1" spans="1:26">
       <c r="A58" s="8">
         <v>58</v>
       </c>
-      <c r="B58" s="41" t="s">
-        <v>185</v>
+      <c r="B58" s="44" t="s">
+        <v>183</v>
       </c>
       <c r="C58" s="19" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D58" s="14">
         <v>415</v>
@@ -6472,11 +6489,11 @@
       <c r="A59" s="8">
         <v>59</v>
       </c>
-      <c r="B59" s="41" t="s">
-        <v>186</v>
+      <c r="B59" s="44" t="s">
+        <v>184</v>
       </c>
       <c r="C59" s="19" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D59" s="21">
         <v>14</v>
@@ -6549,107 +6566,93 @@
       <c r="A60" s="8">
         <v>60</v>
       </c>
-      <c r="B60" s="41" t="s">
-        <v>187</v>
+      <c r="B60" s="44" t="s">
+        <v>185</v>
       </c>
       <c r="C60" s="19"/>
-      <c r="D60" s="51" t="s">
-        <v>165</v>
-      </c>
-      <c r="E60" s="33">
-        <f t="shared" ref="E60" si="0">E59/E11</f>
-        <v>5.38461538461538</v>
-      </c>
-      <c r="F60" s="51" t="s">
-        <v>165</v>
-      </c>
-      <c r="G60" s="33">
-        <f t="shared" ref="G60:Y60" si="1">G59/G11</f>
-        <v>3.55731225296443</v>
-      </c>
-      <c r="H60" s="33">
-        <f t="shared" si="1"/>
-        <v>5.15603799185889</v>
-      </c>
-      <c r="I60" s="33">
-        <f t="shared" si="1"/>
+      <c r="D60" s="54" t="s">
+        <v>164</v>
+      </c>
+      <c r="E60" s="36">
+        <v>5.4</v>
+      </c>
+      <c r="F60" s="54">
+        <v>4.8</v>
+      </c>
+      <c r="G60" s="36">
+        <v>3.6</v>
+      </c>
+      <c r="H60" s="36">
+        <v>5.1</v>
+      </c>
+      <c r="I60" s="36">
+        <f>I59/I11</f>
         <v>3.8</v>
       </c>
-      <c r="J60" s="33">
-        <f t="shared" si="1"/>
-        <v>3.44827586206897</v>
-      </c>
-      <c r="K60" s="33">
-        <f t="shared" si="1"/>
-        <v>3.30578512396694</v>
-      </c>
-      <c r="L60" s="33">
-        <f t="shared" si="1"/>
-        <v>4.16666666666667</v>
-      </c>
-      <c r="M60" s="33">
-        <f t="shared" si="1"/>
-        <v>3.04878048780488</v>
-      </c>
-      <c r="N60" s="33">
-        <f t="shared" si="1"/>
-        <v>2.65734265734266</v>
-      </c>
-      <c r="O60" s="33">
-        <f t="shared" si="1"/>
-        <v>1.95071868583162</v>
-      </c>
-      <c r="P60" s="33">
-        <f t="shared" si="1"/>
+      <c r="J60" s="36">
+        <v>3.4</v>
+      </c>
+      <c r="K60" s="36">
+        <v>3.3</v>
+      </c>
+      <c r="L60" s="36">
+        <v>4.2</v>
+      </c>
+      <c r="M60" s="17">
+        <v>3</v>
+      </c>
+      <c r="N60" s="36">
+        <v>2.6</v>
+      </c>
+      <c r="O60" s="36">
+        <v>1.9</v>
+      </c>
+      <c r="P60" s="36">
+        <f>P59/P11</f>
         <v>2.50417362270451</v>
       </c>
-      <c r="Q60" s="33">
-        <f t="shared" si="1"/>
-        <v>2.10674157303371</v>
-      </c>
-      <c r="R60" s="33">
-        <f t="shared" si="1"/>
-        <v>1.54479917610711</v>
-      </c>
-      <c r="S60" s="33">
-        <f t="shared" si="1"/>
-        <v>2.51361541684122</v>
-      </c>
-      <c r="T60" s="33">
-        <f t="shared" si="1"/>
-        <v>2.06611570247934</v>
-      </c>
-      <c r="U60" s="33">
-        <f t="shared" si="1"/>
-        <v>1.9723865877712</v>
-      </c>
-      <c r="V60" s="33">
-        <f t="shared" si="1"/>
+      <c r="Q60" s="36">
+        <v>2.1</v>
+      </c>
+      <c r="R60" s="36">
+        <v>1.5</v>
+      </c>
+      <c r="S60" s="36">
+        <v>2.5</v>
+      </c>
+      <c r="T60" s="17">
+        <v>2</v>
+      </c>
+      <c r="U60" s="36">
+        <v>1.9</v>
+      </c>
+      <c r="V60" s="36">
+        <f>V59/V11</f>
         <v>2.07770621234157</v>
       </c>
-      <c r="W60" s="33">
-        <f t="shared" si="1"/>
+      <c r="W60" s="36">
+        <f>W59/W11</f>
         <v>1.73130193905817</v>
       </c>
-      <c r="X60" s="33">
-        <f t="shared" si="1"/>
+      <c r="X60" s="36">
+        <f>X59/X11</f>
         <v>1.84266477675408</v>
       </c>
-      <c r="Y60" s="33">
-        <f t="shared" si="1"/>
+      <c r="Y60" s="36">
+        <f>Y59/Y11</f>
         <v>1.5355539806284</v>
       </c>
-      <c r="Z60" s="52"/>
+      <c r="Z60" s="55"/>
     </row>
     <row r="61" customHeight="1" spans="1:26">
       <c r="A61" s="8">
         <v>61</v>
       </c>
-      <c r="B61" s="41" t="s">
-        <v>188</v>
+      <c r="B61" s="44" t="s">
+        <v>186</v>
       </c>
       <c r="C61" s="19" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D61" s="21">
         <v>7</v>
@@ -6722,11 +6725,11 @@
       <c r="A62" s="8">
         <v>62</v>
       </c>
-      <c r="B62" s="41" t="s">
-        <v>190</v>
+      <c r="B62" s="44" t="s">
+        <v>188</v>
       </c>
       <c r="C62" s="19" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D62" s="21">
         <v>0.09</v>
@@ -6800,74 +6803,74 @@
         <v>63</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C63" s="10"/>
       <c r="D63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="I63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="L63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="M63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="N63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="O63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="P63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Q63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="S63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="U63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="V63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="W63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="X63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Y63" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="64" customHeight="1" spans="1:26">
@@ -6875,74 +6878,74 @@
         <v>64</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C64" s="10"/>
-      <c r="D64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="E64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="F64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="G64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="H64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="I64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="J64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="K64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="L64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="M64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="N64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="O64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="P64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="Q64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="R64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="S64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="T64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="U64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="V64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="W64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="X64" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="Y64" s="53" t="s">
-        <v>194</v>
+      <c r="D64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="E64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="F64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="G64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="H64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="I64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="J64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="K64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="L64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="M64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="N64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="O64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="P64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="R64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="S64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="T64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="U64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="V64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="W64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="X64" s="56" t="s">
+        <v>192</v>
+      </c>
+      <c r="Y64" s="56" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="65" customHeight="1" spans="1:25">
@@ -6950,7 +6953,7 @@
         <v>65</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C65" s="10"/>
       <c r="D65" s="20" t="s">
@@ -7025,7 +7028,7 @@
         <v>66</v>
       </c>
       <c r="B66" s="9" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C66" s="10"/>
       <c r="D66" s="20" t="s">
@@ -7100,7 +7103,7 @@
         <v>67</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C67" s="10"/>
       <c r="D67" s="20" t="s">
@@ -7175,7 +7178,7 @@
         <v>68</v>
       </c>
       <c r="B68" s="9" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C68" s="10"/>
       <c r="D68" s="20" t="s">
@@ -7250,7 +7253,7 @@
         <v>69</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C69" s="10"/>
       <c r="D69" s="20" t="s">
@@ -7325,7 +7328,7 @@
         <v>70</v>
       </c>
       <c r="B70" s="9" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C70" s="10"/>
       <c r="D70" s="20" t="s">
@@ -7400,7 +7403,7 @@
         <v>71</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C71" s="10"/>
       <c r="D71" s="20" t="s">

</xml_diff>